<commit_message>
After logging in, a test was written to add a book to favorites.
</commit_message>
<xml_diff>
--- a/AppiumPOM_02/src/test/resources/testdata.xlsx
+++ b/AppiumPOM_02/src/test/resources/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3fab46644dc17b22/Desktop/Appium Examples/AppiumPOM_02/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{65C2C96C-8299-4EE5-900F-AEB22562E785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38DF0474-5596-4ED3-8916-289AA5262225}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{65C2C96C-8299-4EE5-900F-AEB22562E785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6AA5631-BE23-40CB-B294-0B3257C13AE1}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{E0DF160F-E992-4E58-8AC1-1823EDAC366F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{E0DF160F-E992-4E58-8AC1-1823EDAC366F}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Examples were created for TestNG regarding Test Groups and Suite Management. Tests were grouped. Some .xml files were written.
</commit_message>
<xml_diff>
--- a/AppiumPOM_02/src/test/resources/testdata.xlsx
+++ b/AppiumPOM_02/src/test/resources/testdata.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3fab46644dc17b22/Desktop/Appium Examples/AppiumPOM_02/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{65C2C96C-8299-4EE5-900F-AEB22562E785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6AA5631-BE23-40CB-B294-0B3257C13AE1}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="8_{65C2C96C-8299-4EE5-900F-AEB22562E785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B2825AF-6476-4425-A87E-E859EB1801CF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{E0DF160F-E992-4E58-8AC1-1823EDAC366F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{E0DF160F-E992-4E58-8AC1-1823EDAC366F}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
     <sheet name="InvalidLoginData" sheetId="2" r:id="rId2"/>
     <sheet name="ParallelLoginData" sheetId="3" r:id="rId3"/>
+    <sheet name="ParallelLoginData2" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="20">
   <si>
     <t>TestCase</t>
   </si>
@@ -89,6 +90,15 @@
   </si>
   <si>
     <t>wronguserexample.com</t>
+  </si>
+  <si>
+    <t>wronguser2@example.com</t>
+  </si>
+  <si>
+    <t>testuser2@example.com</t>
+  </si>
+  <si>
+    <t>wronguser2example.com</t>
   </si>
 </sst>
 </file>
@@ -131,9 +141,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -660,4 +671,55 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B42465B-E1D4-49CF-9FE1-78BCC9AFD557}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>